<commit_message>
catalog: ม.1–ม.3 activities split into ภาค 1 / ภาค 2
The draft ม.ต้น workbook now lists each activity per semester (84 rows):
codes 01-04 for ภาค 1, 05-08 for ภาค 2, yearly hours unchanged.
Re-importing updates old yearly activity rows in place.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/รายวิชา_ม1-ม3_ฉบับร่าง.xlsx
+++ b/catalog/รายวิชา_ม1-ม3_ฉบับร่าง.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T74"/>
+  <dimension ref="A1:T86"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="9.83203125" customWidth="1"/>
@@ -1794,10 +1794,10 @@
         <v>ก21101</v>
       </c>
       <c r="C23" t="str">
-        <v>แนะแนว</v>
+        <v>แนะแนว 1</v>
       </c>
       <c r="D23">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E23" t="str">
         <v>กิจกรรม</v>
@@ -1844,8 +1844,8 @@
       <c r="S23" t="str">
         <v/>
       </c>
-      <c r="T23" t="str">
-        <v/>
+      <c r="T23">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1853,13 +1853,13 @@
         <v>ม.1</v>
       </c>
       <c r="B24" t="str">
-        <v>ก21102</v>
+        <v>ก21105</v>
       </c>
       <c r="C24" t="str">
-        <v>ลูกเสือ-เนตรนารี</v>
+        <v>แนะแนว 2</v>
       </c>
       <c r="D24">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E24" t="str">
         <v>กิจกรรม</v>
@@ -1906,8 +1906,8 @@
       <c r="S24" t="str">
         <v/>
       </c>
-      <c r="T24" t="str">
-        <v/>
+      <c r="T24">
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -1915,13 +1915,13 @@
         <v>ม.1</v>
       </c>
       <c r="B25" t="str">
-        <v>ก21103</v>
+        <v>ก21102</v>
       </c>
       <c r="C25" t="str">
-        <v>ชุมนุม</v>
+        <v>ลูกเสือ-เนตรนารี 1</v>
       </c>
       <c r="D25">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E25" t="str">
         <v>กิจกรรม</v>
@@ -1968,8 +1968,8 @@
       <c r="S25" t="str">
         <v/>
       </c>
-      <c r="T25" t="str">
-        <v/>
+      <c r="T25">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1977,13 +1977,13 @@
         <v>ม.1</v>
       </c>
       <c r="B26" t="str">
-        <v>ก21104</v>
+        <v>ก21106</v>
       </c>
       <c r="C26" t="str">
-        <v>กิจกรรมเพื่อสังคมและสาธารณประโยชน์</v>
+        <v>ลูกเสือ-เนตรนารี 2</v>
       </c>
       <c r="D26">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E26" t="str">
         <v>กิจกรรม</v>
@@ -2030,61 +2030,61 @@
       <c r="S26" t="str">
         <v/>
       </c>
-      <c r="T26" t="str">
-        <v/>
+      <c r="T26">
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>ม.2</v>
+        <v>ม.1</v>
       </c>
       <c r="B27" t="str">
-        <v>ท22101</v>
+        <v>ก21103</v>
       </c>
       <c r="C27" t="str">
-        <v>ภาษาไทย 1</v>
+        <v>ชุมนุม 1</v>
       </c>
       <c r="D27">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="E27" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F27">
-        <v>5</v>
-      </c>
-      <c r="G27">
-        <v>5</v>
-      </c>
-      <c r="H27">
-        <v>5</v>
-      </c>
-      <c r="I27">
-        <v>10</v>
-      </c>
-      <c r="J27">
-        <v>25</v>
-      </c>
-      <c r="K27">
-        <v>20</v>
-      </c>
-      <c r="L27">
-        <v>5</v>
-      </c>
-      <c r="M27">
-        <v>5</v>
-      </c>
-      <c r="N27">
-        <v>15</v>
-      </c>
-      <c r="O27">
-        <v>25</v>
-      </c>
-      <c r="P27">
-        <v>70</v>
-      </c>
-      <c r="Q27">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F27" t="str">
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
       </c>
       <c r="R27">
         <v>100</v>
@@ -2098,55 +2098,55 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>ม.2</v>
+        <v>ม.1</v>
       </c>
       <c r="B28" t="str">
-        <v>ท22102</v>
+        <v>ก21107</v>
       </c>
       <c r="C28" t="str">
-        <v>ภาษาไทย 2</v>
+        <v>ชุมนุม 2</v>
       </c>
       <c r="D28">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="E28" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F28">
-        <v>5</v>
-      </c>
-      <c r="G28">
-        <v>5</v>
-      </c>
-      <c r="H28">
-        <v>5</v>
-      </c>
-      <c r="I28">
-        <v>10</v>
-      </c>
-      <c r="J28">
-        <v>25</v>
-      </c>
-      <c r="K28">
-        <v>20</v>
-      </c>
-      <c r="L28">
-        <v>5</v>
-      </c>
-      <c r="M28">
-        <v>5</v>
-      </c>
-      <c r="N28">
-        <v>15</v>
-      </c>
-      <c r="O28">
-        <v>25</v>
-      </c>
-      <c r="P28">
-        <v>70</v>
-      </c>
-      <c r="Q28">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
       </c>
       <c r="R28">
         <v>100</v>
@@ -2160,55 +2160,55 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>ม.2</v>
+        <v>ม.1</v>
       </c>
       <c r="B29" t="str">
-        <v>ค22101</v>
+        <v>ก21104</v>
       </c>
       <c r="C29" t="str">
-        <v>คณิตศาสตร์ 1</v>
+        <v>กิจกรรมเพื่อสังคมและสาธารณประโยชน์ 1</v>
       </c>
       <c r="D29">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="E29" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F29">
-        <v>5</v>
-      </c>
-      <c r="G29">
-        <v>5</v>
-      </c>
-      <c r="H29">
-        <v>5</v>
-      </c>
-      <c r="I29">
-        <v>10</v>
-      </c>
-      <c r="J29">
-        <v>25</v>
-      </c>
-      <c r="K29">
-        <v>20</v>
-      </c>
-      <c r="L29">
-        <v>5</v>
-      </c>
-      <c r="M29">
-        <v>5</v>
-      </c>
-      <c r="N29">
-        <v>15</v>
-      </c>
-      <c r="O29">
-        <v>25</v>
-      </c>
-      <c r="P29">
-        <v>70</v>
-      </c>
-      <c r="Q29">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v/>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
       </c>
       <c r="R29">
         <v>100</v>
@@ -2222,55 +2222,55 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>ม.2</v>
+        <v>ม.1</v>
       </c>
       <c r="B30" t="str">
-        <v>ค22102</v>
+        <v>ก21108</v>
       </c>
       <c r="C30" t="str">
-        <v>คณิตศาสตร์ 2</v>
+        <v>กิจกรรมเพื่อสังคมและสาธารณประโยชน์ 2</v>
       </c>
       <c r="D30">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="E30" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F30">
-        <v>5</v>
-      </c>
-      <c r="G30">
-        <v>5</v>
-      </c>
-      <c r="H30">
-        <v>5</v>
-      </c>
-      <c r="I30">
-        <v>10</v>
-      </c>
-      <c r="J30">
-        <v>25</v>
-      </c>
-      <c r="K30">
-        <v>20</v>
-      </c>
-      <c r="L30">
-        <v>5</v>
-      </c>
-      <c r="M30">
-        <v>5</v>
-      </c>
-      <c r="N30">
-        <v>15</v>
-      </c>
-      <c r="O30">
-        <v>25</v>
-      </c>
-      <c r="P30">
-        <v>70</v>
-      </c>
-      <c r="Q30">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v/>
+      </c>
+      <c r="O30" t="str">
+        <v/>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
       </c>
       <c r="R30">
         <v>100</v>
@@ -2287,10 +2287,10 @@
         <v>ม.2</v>
       </c>
       <c r="B31" t="str">
-        <v>ว22101</v>
+        <v>ท22101</v>
       </c>
       <c r="C31" t="str">
-        <v>วิทยาศาสตร์ 1</v>
+        <v>ภาษาไทย 1</v>
       </c>
       <c r="D31">
         <v>60</v>
@@ -2349,10 +2349,10 @@
         <v>ม.2</v>
       </c>
       <c r="B32" t="str">
-        <v>ว22102</v>
+        <v>ท22102</v>
       </c>
       <c r="C32" t="str">
-        <v>วิทยาศาสตร์ 2</v>
+        <v>ภาษาไทย 2</v>
       </c>
       <c r="D32">
         <v>60</v>
@@ -2411,13 +2411,13 @@
         <v>ม.2</v>
       </c>
       <c r="B33" t="str">
-        <v>ว22103</v>
+        <v>ค22101</v>
       </c>
       <c r="C33" t="str">
-        <v>เทคโนโลยี (วิทยาการคำนวณ) 1</v>
+        <v>คณิตศาสตร์ 1</v>
       </c>
       <c r="D33">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E33" t="str">
         <v>พื้นฐาน</v>
@@ -2473,13 +2473,13 @@
         <v>ม.2</v>
       </c>
       <c r="B34" t="str">
-        <v>ว22104</v>
+        <v>ค22102</v>
       </c>
       <c r="C34" t="str">
-        <v>เทคโนโลยี (วิทยาการคำนวณ) 2</v>
+        <v>คณิตศาสตร์ 2</v>
       </c>
       <c r="D34">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E34" t="str">
         <v>พื้นฐาน</v>
@@ -2535,10 +2535,10 @@
         <v>ม.2</v>
       </c>
       <c r="B35" t="str">
-        <v>ส22101</v>
+        <v>ว22101</v>
       </c>
       <c r="C35" t="str">
-        <v>สังคมศึกษา ศาสนา และวัฒนธรรม 1</v>
+        <v>วิทยาศาสตร์ 1</v>
       </c>
       <c r="D35">
         <v>60</v>
@@ -2597,10 +2597,10 @@
         <v>ม.2</v>
       </c>
       <c r="B36" t="str">
-        <v>ส22103</v>
+        <v>ว22102</v>
       </c>
       <c r="C36" t="str">
-        <v>สังคมศึกษา ศาสนา และวัฒนธรรม 2</v>
+        <v>วิทยาศาสตร์ 2</v>
       </c>
       <c r="D36">
         <v>60</v>
@@ -2659,10 +2659,10 @@
         <v>ม.2</v>
       </c>
       <c r="B37" t="str">
-        <v>ส22102</v>
+        <v>ว22103</v>
       </c>
       <c r="C37" t="str">
-        <v>ประวัติศาสตร์ 1</v>
+        <v>เทคโนโลยี (วิทยาการคำนวณ) 1</v>
       </c>
       <c r="D37">
         <v>20</v>
@@ -2721,10 +2721,10 @@
         <v>ม.2</v>
       </c>
       <c r="B38" t="str">
-        <v>ส22104</v>
+        <v>ว22104</v>
       </c>
       <c r="C38" t="str">
-        <v>ประวัติศาสตร์ 2</v>
+        <v>เทคโนโลยี (วิทยาการคำนวณ) 2</v>
       </c>
       <c r="D38">
         <v>20</v>
@@ -2783,13 +2783,13 @@
         <v>ม.2</v>
       </c>
       <c r="B39" t="str">
-        <v>พ22101</v>
+        <v>ส22101</v>
       </c>
       <c r="C39" t="str">
-        <v>สุขศึกษาและพลศึกษา 1</v>
+        <v>สังคมศึกษา ศาสนา และวัฒนธรรม 1</v>
       </c>
       <c r="D39">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E39" t="str">
         <v>พื้นฐาน</v>
@@ -2845,13 +2845,13 @@
         <v>ม.2</v>
       </c>
       <c r="B40" t="str">
-        <v>พ22102</v>
+        <v>ส22103</v>
       </c>
       <c r="C40" t="str">
-        <v>สุขศึกษาและพลศึกษา 2</v>
+        <v>สังคมศึกษา ศาสนา และวัฒนธรรม 2</v>
       </c>
       <c r="D40">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E40" t="str">
         <v>พื้นฐาน</v>
@@ -2907,13 +2907,13 @@
         <v>ม.2</v>
       </c>
       <c r="B41" t="str">
-        <v>ศ22101</v>
+        <v>ส22102</v>
       </c>
       <c r="C41" t="str">
-        <v>ศิลปะ 1</v>
+        <v>ประวัติศาสตร์ 1</v>
       </c>
       <c r="D41">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E41" t="str">
         <v>พื้นฐาน</v>
@@ -2969,13 +2969,13 @@
         <v>ม.2</v>
       </c>
       <c r="B42" t="str">
-        <v>ศ22102</v>
+        <v>ส22104</v>
       </c>
       <c r="C42" t="str">
-        <v>ศิลปะ 2</v>
+        <v>ประวัติศาสตร์ 2</v>
       </c>
       <c r="D42">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E42" t="str">
         <v>พื้นฐาน</v>
@@ -3031,13 +3031,13 @@
         <v>ม.2</v>
       </c>
       <c r="B43" t="str">
-        <v>ง22101</v>
+        <v>พ22101</v>
       </c>
       <c r="C43" t="str">
-        <v>การงานอาชีพ 1</v>
+        <v>สุขศึกษาและพลศึกษา 1</v>
       </c>
       <c r="D43">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E43" t="str">
         <v>พื้นฐาน</v>
@@ -3093,13 +3093,13 @@
         <v>ม.2</v>
       </c>
       <c r="B44" t="str">
-        <v>ง22102</v>
+        <v>พ22102</v>
       </c>
       <c r="C44" t="str">
-        <v>การงานอาชีพ 2</v>
+        <v>สุขศึกษาและพลศึกษา 2</v>
       </c>
       <c r="D44">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="E44" t="str">
         <v>พื้นฐาน</v>
@@ -3155,13 +3155,13 @@
         <v>ม.2</v>
       </c>
       <c r="B45" t="str">
-        <v>อ22101</v>
+        <v>ศ22101</v>
       </c>
       <c r="C45" t="str">
-        <v>ภาษาอังกฤษ 1</v>
+        <v>ศิลปะ 1</v>
       </c>
       <c r="D45">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E45" t="str">
         <v>พื้นฐาน</v>
@@ -3217,13 +3217,13 @@
         <v>ม.2</v>
       </c>
       <c r="B46" t="str">
-        <v>อ22102</v>
+        <v>ศ22102</v>
       </c>
       <c r="C46" t="str">
-        <v>ภาษาอังกฤษ 2</v>
+        <v>ศิลปะ 2</v>
       </c>
       <c r="D46">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E46" t="str">
         <v>พื้นฐาน</v>
@@ -3279,52 +3279,52 @@
         <v>ม.2</v>
       </c>
       <c r="B47" t="str">
-        <v>ก22101</v>
+        <v>ง22101</v>
       </c>
       <c r="C47" t="str">
-        <v>แนะแนว</v>
+        <v>การงานอาชีพ 1</v>
       </c>
       <c r="D47">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E47" t="str">
-        <v>กิจกรรม</v>
-      </c>
-      <c r="F47" t="str">
-        <v/>
-      </c>
-      <c r="G47" t="str">
-        <v/>
-      </c>
-      <c r="H47" t="str">
-        <v/>
-      </c>
-      <c r="I47" t="str">
-        <v/>
-      </c>
-      <c r="J47" t="str">
-        <v/>
-      </c>
-      <c r="K47" t="str">
-        <v/>
-      </c>
-      <c r="L47" t="str">
-        <v/>
-      </c>
-      <c r="M47" t="str">
-        <v/>
-      </c>
-      <c r="N47" t="str">
-        <v/>
-      </c>
-      <c r="O47" t="str">
-        <v/>
-      </c>
-      <c r="P47" t="str">
-        <v/>
-      </c>
-      <c r="Q47" t="str">
-        <v/>
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F47">
+        <v>5</v>
+      </c>
+      <c r="G47">
+        <v>5</v>
+      </c>
+      <c r="H47">
+        <v>5</v>
+      </c>
+      <c r="I47">
+        <v>10</v>
+      </c>
+      <c r="J47">
+        <v>25</v>
+      </c>
+      <c r="K47">
+        <v>20</v>
+      </c>
+      <c r="L47">
+        <v>5</v>
+      </c>
+      <c r="M47">
+        <v>5</v>
+      </c>
+      <c r="N47">
+        <v>15</v>
+      </c>
+      <c r="O47">
+        <v>25</v>
+      </c>
+      <c r="P47">
+        <v>70</v>
+      </c>
+      <c r="Q47">
+        <v>30</v>
       </c>
       <c r="R47">
         <v>100</v>
@@ -3332,8 +3332,8 @@
       <c r="S47" t="str">
         <v/>
       </c>
-      <c r="T47" t="str">
-        <v/>
+      <c r="T47">
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -3341,52 +3341,52 @@
         <v>ม.2</v>
       </c>
       <c r="B48" t="str">
-        <v>ก22102</v>
+        <v>ง22102</v>
       </c>
       <c r="C48" t="str">
-        <v>ลูกเสือ-เนตรนารี</v>
+        <v>การงานอาชีพ 2</v>
       </c>
       <c r="D48">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E48" t="str">
-        <v>กิจกรรม</v>
-      </c>
-      <c r="F48" t="str">
-        <v/>
-      </c>
-      <c r="G48" t="str">
-        <v/>
-      </c>
-      <c r="H48" t="str">
-        <v/>
-      </c>
-      <c r="I48" t="str">
-        <v/>
-      </c>
-      <c r="J48" t="str">
-        <v/>
-      </c>
-      <c r="K48" t="str">
-        <v/>
-      </c>
-      <c r="L48" t="str">
-        <v/>
-      </c>
-      <c r="M48" t="str">
-        <v/>
-      </c>
-      <c r="N48" t="str">
-        <v/>
-      </c>
-      <c r="O48" t="str">
-        <v/>
-      </c>
-      <c r="P48" t="str">
-        <v/>
-      </c>
-      <c r="Q48" t="str">
-        <v/>
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F48">
+        <v>5</v>
+      </c>
+      <c r="G48">
+        <v>5</v>
+      </c>
+      <c r="H48">
+        <v>5</v>
+      </c>
+      <c r="I48">
+        <v>10</v>
+      </c>
+      <c r="J48">
+        <v>25</v>
+      </c>
+      <c r="K48">
+        <v>20</v>
+      </c>
+      <c r="L48">
+        <v>5</v>
+      </c>
+      <c r="M48">
+        <v>5</v>
+      </c>
+      <c r="N48">
+        <v>15</v>
+      </c>
+      <c r="O48">
+        <v>25</v>
+      </c>
+      <c r="P48">
+        <v>70</v>
+      </c>
+      <c r="Q48">
+        <v>30</v>
       </c>
       <c r="R48">
         <v>100</v>
@@ -3394,8 +3394,8 @@
       <c r="S48" t="str">
         <v/>
       </c>
-      <c r="T48" t="str">
-        <v/>
+      <c r="T48">
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -3403,52 +3403,52 @@
         <v>ม.2</v>
       </c>
       <c r="B49" t="str">
-        <v>ก22103</v>
+        <v>อ22101</v>
       </c>
       <c r="C49" t="str">
-        <v>ชุมนุม</v>
+        <v>ภาษาอังกฤษ 1</v>
       </c>
       <c r="D49">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="E49" t="str">
-        <v>กิจกรรม</v>
-      </c>
-      <c r="F49" t="str">
-        <v/>
-      </c>
-      <c r="G49" t="str">
-        <v/>
-      </c>
-      <c r="H49" t="str">
-        <v/>
-      </c>
-      <c r="I49" t="str">
-        <v/>
-      </c>
-      <c r="J49" t="str">
-        <v/>
-      </c>
-      <c r="K49" t="str">
-        <v/>
-      </c>
-      <c r="L49" t="str">
-        <v/>
-      </c>
-      <c r="M49" t="str">
-        <v/>
-      </c>
-      <c r="N49" t="str">
-        <v/>
-      </c>
-      <c r="O49" t="str">
-        <v/>
-      </c>
-      <c r="P49" t="str">
-        <v/>
-      </c>
-      <c r="Q49" t="str">
-        <v/>
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F49">
+        <v>5</v>
+      </c>
+      <c r="G49">
+        <v>5</v>
+      </c>
+      <c r="H49">
+        <v>5</v>
+      </c>
+      <c r="I49">
+        <v>10</v>
+      </c>
+      <c r="J49">
+        <v>25</v>
+      </c>
+      <c r="K49">
+        <v>20</v>
+      </c>
+      <c r="L49">
+        <v>5</v>
+      </c>
+      <c r="M49">
+        <v>5</v>
+      </c>
+      <c r="N49">
+        <v>15</v>
+      </c>
+      <c r="O49">
+        <v>25</v>
+      </c>
+      <c r="P49">
+        <v>70</v>
+      </c>
+      <c r="Q49">
+        <v>30</v>
       </c>
       <c r="R49">
         <v>100</v>
@@ -3456,8 +3456,8 @@
       <c r="S49" t="str">
         <v/>
       </c>
-      <c r="T49" t="str">
-        <v/>
+      <c r="T49">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -3465,52 +3465,52 @@
         <v>ม.2</v>
       </c>
       <c r="B50" t="str">
-        <v>ก22104</v>
+        <v>อ22102</v>
       </c>
       <c r="C50" t="str">
-        <v>กิจกรรมเพื่อสังคมและสาธารณประโยชน์</v>
+        <v>ภาษาอังกฤษ 2</v>
       </c>
       <c r="D50">
+        <v>60</v>
+      </c>
+      <c r="E50" t="str">
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F50">
+        <v>5</v>
+      </c>
+      <c r="G50">
+        <v>5</v>
+      </c>
+      <c r="H50">
+        <v>5</v>
+      </c>
+      <c r="I50">
+        <v>10</v>
+      </c>
+      <c r="J50">
+        <v>25</v>
+      </c>
+      <c r="K50">
+        <v>20</v>
+      </c>
+      <c r="L50">
+        <v>5</v>
+      </c>
+      <c r="M50">
+        <v>5</v>
+      </c>
+      <c r="N50">
         <v>15</v>
       </c>
-      <c r="E50" t="str">
-        <v>กิจกรรม</v>
-      </c>
-      <c r="F50" t="str">
-        <v/>
-      </c>
-      <c r="G50" t="str">
-        <v/>
-      </c>
-      <c r="H50" t="str">
-        <v/>
-      </c>
-      <c r="I50" t="str">
-        <v/>
-      </c>
-      <c r="J50" t="str">
-        <v/>
-      </c>
-      <c r="K50" t="str">
-        <v/>
-      </c>
-      <c r="L50" t="str">
-        <v/>
-      </c>
-      <c r="M50" t="str">
-        <v/>
-      </c>
-      <c r="N50" t="str">
-        <v/>
-      </c>
-      <c r="O50" t="str">
-        <v/>
-      </c>
-      <c r="P50" t="str">
-        <v/>
-      </c>
-      <c r="Q50" t="str">
-        <v/>
+      <c r="O50">
+        <v>25</v>
+      </c>
+      <c r="P50">
+        <v>70</v>
+      </c>
+      <c r="Q50">
+        <v>30</v>
       </c>
       <c r="R50">
         <v>100</v>
@@ -3518,61 +3518,61 @@
       <c r="S50" t="str">
         <v/>
       </c>
-      <c r="T50" t="str">
-        <v/>
+      <c r="T50">
+        <v>2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>ม.3</v>
+        <v>ม.2</v>
       </c>
       <c r="B51" t="str">
-        <v>ท23101</v>
+        <v>ก22101</v>
       </c>
       <c r="C51" t="str">
-        <v>ภาษาไทย 1</v>
+        <v>แนะแนว 1</v>
       </c>
       <c r="D51">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E51" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F51">
-        <v>5</v>
-      </c>
-      <c r="G51">
-        <v>5</v>
-      </c>
-      <c r="H51">
-        <v>5</v>
-      </c>
-      <c r="I51">
-        <v>10</v>
-      </c>
-      <c r="J51">
-        <v>25</v>
-      </c>
-      <c r="K51">
-        <v>20</v>
-      </c>
-      <c r="L51">
-        <v>5</v>
-      </c>
-      <c r="M51">
-        <v>5</v>
-      </c>
-      <c r="N51">
-        <v>15</v>
-      </c>
-      <c r="O51">
-        <v>25</v>
-      </c>
-      <c r="P51">
-        <v>70</v>
-      </c>
-      <c r="Q51">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+      <c r="K51" t="str">
+        <v/>
+      </c>
+      <c r="L51" t="str">
+        <v/>
+      </c>
+      <c r="M51" t="str">
+        <v/>
+      </c>
+      <c r="N51" t="str">
+        <v/>
+      </c>
+      <c r="O51" t="str">
+        <v/>
+      </c>
+      <c r="P51" t="str">
+        <v/>
+      </c>
+      <c r="Q51" t="str">
+        <v/>
       </c>
       <c r="R51">
         <v>100</v>
@@ -3586,55 +3586,55 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>ม.3</v>
+        <v>ม.2</v>
       </c>
       <c r="B52" t="str">
-        <v>ท23102</v>
+        <v>ก22105</v>
       </c>
       <c r="C52" t="str">
-        <v>ภาษาไทย 2</v>
+        <v>แนะแนว 2</v>
       </c>
       <c r="D52">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E52" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F52">
-        <v>5</v>
-      </c>
-      <c r="G52">
-        <v>5</v>
-      </c>
-      <c r="H52">
-        <v>5</v>
-      </c>
-      <c r="I52">
-        <v>10</v>
-      </c>
-      <c r="J52">
-        <v>25</v>
-      </c>
-      <c r="K52">
-        <v>20</v>
-      </c>
-      <c r="L52">
-        <v>5</v>
-      </c>
-      <c r="M52">
-        <v>5</v>
-      </c>
-      <c r="N52">
-        <v>15</v>
-      </c>
-      <c r="O52">
-        <v>25</v>
-      </c>
-      <c r="P52">
-        <v>70</v>
-      </c>
-      <c r="Q52">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
+        <v/>
+      </c>
+      <c r="L52" t="str">
+        <v/>
+      </c>
+      <c r="M52" t="str">
+        <v/>
+      </c>
+      <c r="N52" t="str">
+        <v/>
+      </c>
+      <c r="O52" t="str">
+        <v/>
+      </c>
+      <c r="P52" t="str">
+        <v/>
+      </c>
+      <c r="Q52" t="str">
+        <v/>
       </c>
       <c r="R52">
         <v>100</v>
@@ -3648,55 +3648,55 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>ม.3</v>
+        <v>ม.2</v>
       </c>
       <c r="B53" t="str">
-        <v>ค23101</v>
+        <v>ก22102</v>
       </c>
       <c r="C53" t="str">
-        <v>คณิตศาสตร์ 1</v>
+        <v>ลูกเสือ-เนตรนารี 1</v>
       </c>
       <c r="D53">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E53" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F53">
-        <v>5</v>
-      </c>
-      <c r="G53">
-        <v>5</v>
-      </c>
-      <c r="H53">
-        <v>5</v>
-      </c>
-      <c r="I53">
-        <v>10</v>
-      </c>
-      <c r="J53">
-        <v>25</v>
-      </c>
-      <c r="K53">
-        <v>20</v>
-      </c>
-      <c r="L53">
-        <v>5</v>
-      </c>
-      <c r="M53">
-        <v>5</v>
-      </c>
-      <c r="N53">
-        <v>15</v>
-      </c>
-      <c r="O53">
-        <v>25</v>
-      </c>
-      <c r="P53">
-        <v>70</v>
-      </c>
-      <c r="Q53">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+      <c r="K53" t="str">
+        <v/>
+      </c>
+      <c r="L53" t="str">
+        <v/>
+      </c>
+      <c r="M53" t="str">
+        <v/>
+      </c>
+      <c r="N53" t="str">
+        <v/>
+      </c>
+      <c r="O53" t="str">
+        <v/>
+      </c>
+      <c r="P53" t="str">
+        <v/>
+      </c>
+      <c r="Q53" t="str">
+        <v/>
       </c>
       <c r="R53">
         <v>100</v>
@@ -3710,55 +3710,55 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>ม.3</v>
+        <v>ม.2</v>
       </c>
       <c r="B54" t="str">
-        <v>ค23102</v>
+        <v>ก22106</v>
       </c>
       <c r="C54" t="str">
-        <v>คณิตศาสตร์ 2</v>
+        <v>ลูกเสือ-เนตรนารี 2</v>
       </c>
       <c r="D54">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E54" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F54">
-        <v>5</v>
-      </c>
-      <c r="G54">
-        <v>5</v>
-      </c>
-      <c r="H54">
-        <v>5</v>
-      </c>
-      <c r="I54">
-        <v>10</v>
-      </c>
-      <c r="J54">
-        <v>25</v>
-      </c>
-      <c r="K54">
-        <v>20</v>
-      </c>
-      <c r="L54">
-        <v>5</v>
-      </c>
-      <c r="M54">
-        <v>5</v>
-      </c>
-      <c r="N54">
-        <v>15</v>
-      </c>
-      <c r="O54">
-        <v>25</v>
-      </c>
-      <c r="P54">
-        <v>70</v>
-      </c>
-      <c r="Q54">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+      <c r="K54" t="str">
+        <v/>
+      </c>
+      <c r="L54" t="str">
+        <v/>
+      </c>
+      <c r="M54" t="str">
+        <v/>
+      </c>
+      <c r="N54" t="str">
+        <v/>
+      </c>
+      <c r="O54" t="str">
+        <v/>
+      </c>
+      <c r="P54" t="str">
+        <v/>
+      </c>
+      <c r="Q54" t="str">
+        <v/>
       </c>
       <c r="R54">
         <v>100</v>
@@ -3772,55 +3772,55 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>ม.3</v>
+        <v>ม.2</v>
       </c>
       <c r="B55" t="str">
-        <v>ว23101</v>
+        <v>ก22103</v>
       </c>
       <c r="C55" t="str">
-        <v>วิทยาศาสตร์ 1</v>
+        <v>ชุมนุม 1</v>
       </c>
       <c r="D55">
-        <v>60</v>
+        <v>13</v>
       </c>
       <c r="E55" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F55">
-        <v>5</v>
-      </c>
-      <c r="G55">
-        <v>5</v>
-      </c>
-      <c r="H55">
-        <v>5</v>
-      </c>
-      <c r="I55">
-        <v>10</v>
-      </c>
-      <c r="J55">
-        <v>25</v>
-      </c>
-      <c r="K55">
-        <v>20</v>
-      </c>
-      <c r="L55">
-        <v>5</v>
-      </c>
-      <c r="M55">
-        <v>5</v>
-      </c>
-      <c r="N55">
-        <v>15</v>
-      </c>
-      <c r="O55">
-        <v>25</v>
-      </c>
-      <c r="P55">
-        <v>70</v>
-      </c>
-      <c r="Q55">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+      <c r="K55" t="str">
+        <v/>
+      </c>
+      <c r="L55" t="str">
+        <v/>
+      </c>
+      <c r="M55" t="str">
+        <v/>
+      </c>
+      <c r="N55" t="str">
+        <v/>
+      </c>
+      <c r="O55" t="str">
+        <v/>
+      </c>
+      <c r="P55" t="str">
+        <v/>
+      </c>
+      <c r="Q55" t="str">
+        <v/>
       </c>
       <c r="R55">
         <v>100</v>
@@ -3834,55 +3834,55 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>ม.3</v>
+        <v>ม.2</v>
       </c>
       <c r="B56" t="str">
-        <v>ว23102</v>
+        <v>ก22107</v>
       </c>
       <c r="C56" t="str">
-        <v>วิทยาศาสตร์ 2</v>
+        <v>ชุมนุม 2</v>
       </c>
       <c r="D56">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="E56" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F56">
-        <v>5</v>
-      </c>
-      <c r="G56">
-        <v>5</v>
-      </c>
-      <c r="H56">
-        <v>5</v>
-      </c>
-      <c r="I56">
-        <v>10</v>
-      </c>
-      <c r="J56">
-        <v>25</v>
-      </c>
-      <c r="K56">
-        <v>20</v>
-      </c>
-      <c r="L56">
-        <v>5</v>
-      </c>
-      <c r="M56">
-        <v>5</v>
-      </c>
-      <c r="N56">
-        <v>15</v>
-      </c>
-      <c r="O56">
-        <v>25</v>
-      </c>
-      <c r="P56">
-        <v>70</v>
-      </c>
-      <c r="Q56">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+      <c r="K56" t="str">
+        <v/>
+      </c>
+      <c r="L56" t="str">
+        <v/>
+      </c>
+      <c r="M56" t="str">
+        <v/>
+      </c>
+      <c r="N56" t="str">
+        <v/>
+      </c>
+      <c r="O56" t="str">
+        <v/>
+      </c>
+      <c r="P56" t="str">
+        <v/>
+      </c>
+      <c r="Q56" t="str">
+        <v/>
       </c>
       <c r="R56">
         <v>100</v>
@@ -3896,55 +3896,55 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>ม.3</v>
+        <v>ม.2</v>
       </c>
       <c r="B57" t="str">
-        <v>ว23103</v>
+        <v>ก22104</v>
       </c>
       <c r="C57" t="str">
-        <v>เทคโนโลยี (วิทยาการคำนวณ) 1</v>
+        <v>กิจกรรมเพื่อสังคมและสาธารณประโยชน์ 1</v>
       </c>
       <c r="D57">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E57" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F57">
-        <v>5</v>
-      </c>
-      <c r="G57">
-        <v>5</v>
-      </c>
-      <c r="H57">
-        <v>5</v>
-      </c>
-      <c r="I57">
-        <v>10</v>
-      </c>
-      <c r="J57">
-        <v>25</v>
-      </c>
-      <c r="K57">
-        <v>20</v>
-      </c>
-      <c r="L57">
-        <v>5</v>
-      </c>
-      <c r="M57">
-        <v>5</v>
-      </c>
-      <c r="N57">
-        <v>15</v>
-      </c>
-      <c r="O57">
-        <v>25</v>
-      </c>
-      <c r="P57">
-        <v>70</v>
-      </c>
-      <c r="Q57">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+      <c r="K57" t="str">
+        <v/>
+      </c>
+      <c r="L57" t="str">
+        <v/>
+      </c>
+      <c r="M57" t="str">
+        <v/>
+      </c>
+      <c r="N57" t="str">
+        <v/>
+      </c>
+      <c r="O57" t="str">
+        <v/>
+      </c>
+      <c r="P57" t="str">
+        <v/>
+      </c>
+      <c r="Q57" t="str">
+        <v/>
       </c>
       <c r="R57">
         <v>100</v>
@@ -3958,55 +3958,55 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>ม.3</v>
+        <v>ม.2</v>
       </c>
       <c r="B58" t="str">
-        <v>ว23104</v>
+        <v>ก22108</v>
       </c>
       <c r="C58" t="str">
-        <v>เทคโนโลยี (วิทยาการคำนวณ) 2</v>
+        <v>กิจกรรมเพื่อสังคมและสาธารณประโยชน์ 2</v>
       </c>
       <c r="D58">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="E58" t="str">
-        <v>พื้นฐาน</v>
-      </c>
-      <c r="F58">
-        <v>5</v>
-      </c>
-      <c r="G58">
-        <v>5</v>
-      </c>
-      <c r="H58">
-        <v>5</v>
-      </c>
-      <c r="I58">
-        <v>10</v>
-      </c>
-      <c r="J58">
-        <v>25</v>
-      </c>
-      <c r="K58">
-        <v>20</v>
-      </c>
-      <c r="L58">
-        <v>5</v>
-      </c>
-      <c r="M58">
-        <v>5</v>
-      </c>
-      <c r="N58">
-        <v>15</v>
-      </c>
-      <c r="O58">
-        <v>25</v>
-      </c>
-      <c r="P58">
-        <v>70</v>
-      </c>
-      <c r="Q58">
-        <v>30</v>
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+      <c r="K58" t="str">
+        <v/>
+      </c>
+      <c r="L58" t="str">
+        <v/>
+      </c>
+      <c r="M58" t="str">
+        <v/>
+      </c>
+      <c r="N58" t="str">
+        <v/>
+      </c>
+      <c r="O58" t="str">
+        <v/>
+      </c>
+      <c r="P58" t="str">
+        <v/>
+      </c>
+      <c r="Q58" t="str">
+        <v/>
       </c>
       <c r="R58">
         <v>100</v>
@@ -4023,10 +4023,10 @@
         <v>ม.3</v>
       </c>
       <c r="B59" t="str">
-        <v>ส23101</v>
+        <v>ท23101</v>
       </c>
       <c r="C59" t="str">
-        <v>สังคมศึกษา ศาสนา และวัฒนธรรม 1</v>
+        <v>ภาษาไทย 1</v>
       </c>
       <c r="D59">
         <v>60</v>
@@ -4085,10 +4085,10 @@
         <v>ม.3</v>
       </c>
       <c r="B60" t="str">
-        <v>ส23103</v>
+        <v>ท23102</v>
       </c>
       <c r="C60" t="str">
-        <v>สังคมศึกษา ศาสนา และวัฒนธรรม 2</v>
+        <v>ภาษาไทย 2</v>
       </c>
       <c r="D60">
         <v>60</v>
@@ -4147,13 +4147,13 @@
         <v>ม.3</v>
       </c>
       <c r="B61" t="str">
-        <v>ส23102</v>
+        <v>ค23101</v>
       </c>
       <c r="C61" t="str">
-        <v>ประวัติศาสตร์ 1</v>
+        <v>คณิตศาสตร์ 1</v>
       </c>
       <c r="D61">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E61" t="str">
         <v>พื้นฐาน</v>
@@ -4209,13 +4209,13 @@
         <v>ม.3</v>
       </c>
       <c r="B62" t="str">
-        <v>ส23104</v>
+        <v>ค23102</v>
       </c>
       <c r="C62" t="str">
-        <v>ประวัติศาสตร์ 2</v>
+        <v>คณิตศาสตร์ 2</v>
       </c>
       <c r="D62">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E62" t="str">
         <v>พื้นฐาน</v>
@@ -4271,13 +4271,13 @@
         <v>ม.3</v>
       </c>
       <c r="B63" t="str">
-        <v>พ23101</v>
+        <v>ว23101</v>
       </c>
       <c r="C63" t="str">
-        <v>สุขศึกษาและพลศึกษา 1</v>
+        <v>วิทยาศาสตร์ 1</v>
       </c>
       <c r="D63">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E63" t="str">
         <v>พื้นฐาน</v>
@@ -4333,13 +4333,13 @@
         <v>ม.3</v>
       </c>
       <c r="B64" t="str">
-        <v>พ23102</v>
+        <v>ว23102</v>
       </c>
       <c r="C64" t="str">
-        <v>สุขศึกษาและพลศึกษา 2</v>
+        <v>วิทยาศาสตร์ 2</v>
       </c>
       <c r="D64">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E64" t="str">
         <v>พื้นฐาน</v>
@@ -4395,13 +4395,13 @@
         <v>ม.3</v>
       </c>
       <c r="B65" t="str">
-        <v>ศ23101</v>
+        <v>ว23103</v>
       </c>
       <c r="C65" t="str">
-        <v>ศิลปะ 1</v>
+        <v>เทคโนโลยี (วิทยาการคำนวณ) 1</v>
       </c>
       <c r="D65">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E65" t="str">
         <v>พื้นฐาน</v>
@@ -4457,13 +4457,13 @@
         <v>ม.3</v>
       </c>
       <c r="B66" t="str">
-        <v>ศ23102</v>
+        <v>ว23104</v>
       </c>
       <c r="C66" t="str">
-        <v>ศิลปะ 2</v>
+        <v>เทคโนโลยี (วิทยาการคำนวณ) 2</v>
       </c>
       <c r="D66">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E66" t="str">
         <v>พื้นฐาน</v>
@@ -4519,13 +4519,13 @@
         <v>ม.3</v>
       </c>
       <c r="B67" t="str">
-        <v>ง23101</v>
+        <v>ส23101</v>
       </c>
       <c r="C67" t="str">
-        <v>การงานอาชีพ 1</v>
+        <v>สังคมศึกษา ศาสนา และวัฒนธรรม 1</v>
       </c>
       <c r="D67">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E67" t="str">
         <v>พื้นฐาน</v>
@@ -4581,13 +4581,13 @@
         <v>ม.3</v>
       </c>
       <c r="B68" t="str">
-        <v>ง23102</v>
+        <v>ส23103</v>
       </c>
       <c r="C68" t="str">
-        <v>การงานอาชีพ 2</v>
+        <v>สังคมศึกษา ศาสนา และวัฒนธรรม 2</v>
       </c>
       <c r="D68">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E68" t="str">
         <v>พื้นฐาน</v>
@@ -4643,13 +4643,13 @@
         <v>ม.3</v>
       </c>
       <c r="B69" t="str">
-        <v>อ23101</v>
+        <v>ส23102</v>
       </c>
       <c r="C69" t="str">
-        <v>ภาษาอังกฤษ 1</v>
+        <v>ประวัติศาสตร์ 1</v>
       </c>
       <c r="D69">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E69" t="str">
         <v>พื้นฐาน</v>
@@ -4705,13 +4705,13 @@
         <v>ม.3</v>
       </c>
       <c r="B70" t="str">
-        <v>อ23102</v>
+        <v>ส23104</v>
       </c>
       <c r="C70" t="str">
-        <v>ภาษาอังกฤษ 2</v>
+        <v>ประวัติศาสตร์ 2</v>
       </c>
       <c r="D70">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E70" t="str">
         <v>พื้นฐาน</v>
@@ -4767,52 +4767,52 @@
         <v>ม.3</v>
       </c>
       <c r="B71" t="str">
-        <v>ก23101</v>
+        <v>พ23101</v>
       </c>
       <c r="C71" t="str">
-        <v>แนะแนว</v>
+        <v>สุขศึกษาและพลศึกษา 1</v>
       </c>
       <c r="D71">
         <v>40</v>
       </c>
       <c r="E71" t="str">
-        <v>กิจกรรม</v>
-      </c>
-      <c r="F71" t="str">
-        <v/>
-      </c>
-      <c r="G71" t="str">
-        <v/>
-      </c>
-      <c r="H71" t="str">
-        <v/>
-      </c>
-      <c r="I71" t="str">
-        <v/>
-      </c>
-      <c r="J71" t="str">
-        <v/>
-      </c>
-      <c r="K71" t="str">
-        <v/>
-      </c>
-      <c r="L71" t="str">
-        <v/>
-      </c>
-      <c r="M71" t="str">
-        <v/>
-      </c>
-      <c r="N71" t="str">
-        <v/>
-      </c>
-      <c r="O71" t="str">
-        <v/>
-      </c>
-      <c r="P71" t="str">
-        <v/>
-      </c>
-      <c r="Q71" t="str">
-        <v/>
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F71">
+        <v>5</v>
+      </c>
+      <c r="G71">
+        <v>5</v>
+      </c>
+      <c r="H71">
+        <v>5</v>
+      </c>
+      <c r="I71">
+        <v>10</v>
+      </c>
+      <c r="J71">
+        <v>25</v>
+      </c>
+      <c r="K71">
+        <v>20</v>
+      </c>
+      <c r="L71">
+        <v>5</v>
+      </c>
+      <c r="M71">
+        <v>5</v>
+      </c>
+      <c r="N71">
+        <v>15</v>
+      </c>
+      <c r="O71">
+        <v>25</v>
+      </c>
+      <c r="P71">
+        <v>70</v>
+      </c>
+      <c r="Q71">
+        <v>30</v>
       </c>
       <c r="R71">
         <v>100</v>
@@ -4820,8 +4820,8 @@
       <c r="S71" t="str">
         <v/>
       </c>
-      <c r="T71" t="str">
-        <v/>
+      <c r="T71">
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -4829,52 +4829,52 @@
         <v>ม.3</v>
       </c>
       <c r="B72" t="str">
-        <v>ก23102</v>
+        <v>พ23102</v>
       </c>
       <c r="C72" t="str">
-        <v>ลูกเสือ-เนตรนารี</v>
+        <v>สุขศึกษาและพลศึกษา 2</v>
       </c>
       <c r="D72">
         <v>40</v>
       </c>
       <c r="E72" t="str">
-        <v>กิจกรรม</v>
-      </c>
-      <c r="F72" t="str">
-        <v/>
-      </c>
-      <c r="G72" t="str">
-        <v/>
-      </c>
-      <c r="H72" t="str">
-        <v/>
-      </c>
-      <c r="I72" t="str">
-        <v/>
-      </c>
-      <c r="J72" t="str">
-        <v/>
-      </c>
-      <c r="K72" t="str">
-        <v/>
-      </c>
-      <c r="L72" t="str">
-        <v/>
-      </c>
-      <c r="M72" t="str">
-        <v/>
-      </c>
-      <c r="N72" t="str">
-        <v/>
-      </c>
-      <c r="O72" t="str">
-        <v/>
-      </c>
-      <c r="P72" t="str">
-        <v/>
-      </c>
-      <c r="Q72" t="str">
-        <v/>
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F72">
+        <v>5</v>
+      </c>
+      <c r="G72">
+        <v>5</v>
+      </c>
+      <c r="H72">
+        <v>5</v>
+      </c>
+      <c r="I72">
+        <v>10</v>
+      </c>
+      <c r="J72">
+        <v>25</v>
+      </c>
+      <c r="K72">
+        <v>20</v>
+      </c>
+      <c r="L72">
+        <v>5</v>
+      </c>
+      <c r="M72">
+        <v>5</v>
+      </c>
+      <c r="N72">
+        <v>15</v>
+      </c>
+      <c r="O72">
+        <v>25</v>
+      </c>
+      <c r="P72">
+        <v>70</v>
+      </c>
+      <c r="Q72">
+        <v>30</v>
       </c>
       <c r="R72">
         <v>100</v>
@@ -4882,8 +4882,8 @@
       <c r="S72" t="str">
         <v/>
       </c>
-      <c r="T72" t="str">
-        <v/>
+      <c r="T72">
+        <v>2</v>
       </c>
     </row>
     <row r="73">
@@ -4891,52 +4891,52 @@
         <v>ม.3</v>
       </c>
       <c r="B73" t="str">
-        <v>ก23103</v>
+        <v>ศ23101</v>
       </c>
       <c r="C73" t="str">
-        <v>ชุมนุม</v>
+        <v>ศิลปะ 1</v>
       </c>
       <c r="D73">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E73" t="str">
-        <v>กิจกรรม</v>
-      </c>
-      <c r="F73" t="str">
-        <v/>
-      </c>
-      <c r="G73" t="str">
-        <v/>
-      </c>
-      <c r="H73" t="str">
-        <v/>
-      </c>
-      <c r="I73" t="str">
-        <v/>
-      </c>
-      <c r="J73" t="str">
-        <v/>
-      </c>
-      <c r="K73" t="str">
-        <v/>
-      </c>
-      <c r="L73" t="str">
-        <v/>
-      </c>
-      <c r="M73" t="str">
-        <v/>
-      </c>
-      <c r="N73" t="str">
-        <v/>
-      </c>
-      <c r="O73" t="str">
-        <v/>
-      </c>
-      <c r="P73" t="str">
-        <v/>
-      </c>
-      <c r="Q73" t="str">
-        <v/>
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F73">
+        <v>5</v>
+      </c>
+      <c r="G73">
+        <v>5</v>
+      </c>
+      <c r="H73">
+        <v>5</v>
+      </c>
+      <c r="I73">
+        <v>10</v>
+      </c>
+      <c r="J73">
+        <v>25</v>
+      </c>
+      <c r="K73">
+        <v>20</v>
+      </c>
+      <c r="L73">
+        <v>5</v>
+      </c>
+      <c r="M73">
+        <v>5</v>
+      </c>
+      <c r="N73">
+        <v>15</v>
+      </c>
+      <c r="O73">
+        <v>25</v>
+      </c>
+      <c r="P73">
+        <v>70</v>
+      </c>
+      <c r="Q73">
+        <v>30</v>
       </c>
       <c r="R73">
         <v>100</v>
@@ -4944,8 +4944,8 @@
       <c r="S73" t="str">
         <v/>
       </c>
-      <c r="T73" t="str">
-        <v/>
+      <c r="T73">
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -4953,61 +4953,805 @@
         <v>ม.3</v>
       </c>
       <c r="B74" t="str">
+        <v>ศ23102</v>
+      </c>
+      <c r="C74" t="str">
+        <v>ศิลปะ 2</v>
+      </c>
+      <c r="D74">
+        <v>40</v>
+      </c>
+      <c r="E74" t="str">
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F74">
+        <v>5</v>
+      </c>
+      <c r="G74">
+        <v>5</v>
+      </c>
+      <c r="H74">
+        <v>5</v>
+      </c>
+      <c r="I74">
+        <v>10</v>
+      </c>
+      <c r="J74">
+        <v>25</v>
+      </c>
+      <c r="K74">
+        <v>20</v>
+      </c>
+      <c r="L74">
+        <v>5</v>
+      </c>
+      <c r="M74">
+        <v>5</v>
+      </c>
+      <c r="N74">
+        <v>15</v>
+      </c>
+      <c r="O74">
+        <v>25</v>
+      </c>
+      <c r="P74">
+        <v>70</v>
+      </c>
+      <c r="Q74">
+        <v>30</v>
+      </c>
+      <c r="R74">
+        <v>100</v>
+      </c>
+      <c r="S74" t="str">
+        <v/>
+      </c>
+      <c r="T74">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B75" t="str">
+        <v>ง23101</v>
+      </c>
+      <c r="C75" t="str">
+        <v>การงานอาชีพ 1</v>
+      </c>
+      <c r="D75">
+        <v>20</v>
+      </c>
+      <c r="E75" t="str">
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F75">
+        <v>5</v>
+      </c>
+      <c r="G75">
+        <v>5</v>
+      </c>
+      <c r="H75">
+        <v>5</v>
+      </c>
+      <c r="I75">
+        <v>10</v>
+      </c>
+      <c r="J75">
+        <v>25</v>
+      </c>
+      <c r="K75">
+        <v>20</v>
+      </c>
+      <c r="L75">
+        <v>5</v>
+      </c>
+      <c r="M75">
+        <v>5</v>
+      </c>
+      <c r="N75">
+        <v>15</v>
+      </c>
+      <c r="O75">
+        <v>25</v>
+      </c>
+      <c r="P75">
+        <v>70</v>
+      </c>
+      <c r="Q75">
+        <v>30</v>
+      </c>
+      <c r="R75">
+        <v>100</v>
+      </c>
+      <c r="S75" t="str">
+        <v/>
+      </c>
+      <c r="T75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B76" t="str">
+        <v>ง23102</v>
+      </c>
+      <c r="C76" t="str">
+        <v>การงานอาชีพ 2</v>
+      </c>
+      <c r="D76">
+        <v>20</v>
+      </c>
+      <c r="E76" t="str">
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F76">
+        <v>5</v>
+      </c>
+      <c r="G76">
+        <v>5</v>
+      </c>
+      <c r="H76">
+        <v>5</v>
+      </c>
+      <c r="I76">
+        <v>10</v>
+      </c>
+      <c r="J76">
+        <v>25</v>
+      </c>
+      <c r="K76">
+        <v>20</v>
+      </c>
+      <c r="L76">
+        <v>5</v>
+      </c>
+      <c r="M76">
+        <v>5</v>
+      </c>
+      <c r="N76">
+        <v>15</v>
+      </c>
+      <c r="O76">
+        <v>25</v>
+      </c>
+      <c r="P76">
+        <v>70</v>
+      </c>
+      <c r="Q76">
+        <v>30</v>
+      </c>
+      <c r="R76">
+        <v>100</v>
+      </c>
+      <c r="S76" t="str">
+        <v/>
+      </c>
+      <c r="T76">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B77" t="str">
+        <v>อ23101</v>
+      </c>
+      <c r="C77" t="str">
+        <v>ภาษาอังกฤษ 1</v>
+      </c>
+      <c r="D77">
+        <v>60</v>
+      </c>
+      <c r="E77" t="str">
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F77">
+        <v>5</v>
+      </c>
+      <c r="G77">
+        <v>5</v>
+      </c>
+      <c r="H77">
+        <v>5</v>
+      </c>
+      <c r="I77">
+        <v>10</v>
+      </c>
+      <c r="J77">
+        <v>25</v>
+      </c>
+      <c r="K77">
+        <v>20</v>
+      </c>
+      <c r="L77">
+        <v>5</v>
+      </c>
+      <c r="M77">
+        <v>5</v>
+      </c>
+      <c r="N77">
+        <v>15</v>
+      </c>
+      <c r="O77">
+        <v>25</v>
+      </c>
+      <c r="P77">
+        <v>70</v>
+      </c>
+      <c r="Q77">
+        <v>30</v>
+      </c>
+      <c r="R77">
+        <v>100</v>
+      </c>
+      <c r="S77" t="str">
+        <v/>
+      </c>
+      <c r="T77">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B78" t="str">
+        <v>อ23102</v>
+      </c>
+      <c r="C78" t="str">
+        <v>ภาษาอังกฤษ 2</v>
+      </c>
+      <c r="D78">
+        <v>60</v>
+      </c>
+      <c r="E78" t="str">
+        <v>พื้นฐาน</v>
+      </c>
+      <c r="F78">
+        <v>5</v>
+      </c>
+      <c r="G78">
+        <v>5</v>
+      </c>
+      <c r="H78">
+        <v>5</v>
+      </c>
+      <c r="I78">
+        <v>10</v>
+      </c>
+      <c r="J78">
+        <v>25</v>
+      </c>
+      <c r="K78">
+        <v>20</v>
+      </c>
+      <c r="L78">
+        <v>5</v>
+      </c>
+      <c r="M78">
+        <v>5</v>
+      </c>
+      <c r="N78">
+        <v>15</v>
+      </c>
+      <c r="O78">
+        <v>25</v>
+      </c>
+      <c r="P78">
+        <v>70</v>
+      </c>
+      <c r="Q78">
+        <v>30</v>
+      </c>
+      <c r="R78">
+        <v>100</v>
+      </c>
+      <c r="S78" t="str">
+        <v/>
+      </c>
+      <c r="T78">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B79" t="str">
+        <v>ก23101</v>
+      </c>
+      <c r="C79" t="str">
+        <v>แนะแนว 1</v>
+      </c>
+      <c r="D79">
+        <v>20</v>
+      </c>
+      <c r="E79" t="str">
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F79" t="str">
+        <v/>
+      </c>
+      <c r="G79" t="str">
+        <v/>
+      </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
+      <c r="I79" t="str">
+        <v/>
+      </c>
+      <c r="J79" t="str">
+        <v/>
+      </c>
+      <c r="K79" t="str">
+        <v/>
+      </c>
+      <c r="L79" t="str">
+        <v/>
+      </c>
+      <c r="M79" t="str">
+        <v/>
+      </c>
+      <c r="N79" t="str">
+        <v/>
+      </c>
+      <c r="O79" t="str">
+        <v/>
+      </c>
+      <c r="P79" t="str">
+        <v/>
+      </c>
+      <c r="Q79" t="str">
+        <v/>
+      </c>
+      <c r="R79">
+        <v>100</v>
+      </c>
+      <c r="S79" t="str">
+        <v/>
+      </c>
+      <c r="T79">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B80" t="str">
+        <v>ก23105</v>
+      </c>
+      <c r="C80" t="str">
+        <v>แนะแนว 2</v>
+      </c>
+      <c r="D80">
+        <v>20</v>
+      </c>
+      <c r="E80" t="str">
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
+      <c r="H80" t="str">
+        <v/>
+      </c>
+      <c r="I80" t="str">
+        <v/>
+      </c>
+      <c r="J80" t="str">
+        <v/>
+      </c>
+      <c r="K80" t="str">
+        <v/>
+      </c>
+      <c r="L80" t="str">
+        <v/>
+      </c>
+      <c r="M80" t="str">
+        <v/>
+      </c>
+      <c r="N80" t="str">
+        <v/>
+      </c>
+      <c r="O80" t="str">
+        <v/>
+      </c>
+      <c r="P80" t="str">
+        <v/>
+      </c>
+      <c r="Q80" t="str">
+        <v/>
+      </c>
+      <c r="R80">
+        <v>100</v>
+      </c>
+      <c r="S80" t="str">
+        <v/>
+      </c>
+      <c r="T80">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B81" t="str">
+        <v>ก23102</v>
+      </c>
+      <c r="C81" t="str">
+        <v>ลูกเสือ-เนตรนารี 1</v>
+      </c>
+      <c r="D81">
+        <v>20</v>
+      </c>
+      <c r="E81" t="str">
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+      <c r="G81" t="str">
+        <v/>
+      </c>
+      <c r="H81" t="str">
+        <v/>
+      </c>
+      <c r="I81" t="str">
+        <v/>
+      </c>
+      <c r="J81" t="str">
+        <v/>
+      </c>
+      <c r="K81" t="str">
+        <v/>
+      </c>
+      <c r="L81" t="str">
+        <v/>
+      </c>
+      <c r="M81" t="str">
+        <v/>
+      </c>
+      <c r="N81" t="str">
+        <v/>
+      </c>
+      <c r="O81" t="str">
+        <v/>
+      </c>
+      <c r="P81" t="str">
+        <v/>
+      </c>
+      <c r="Q81" t="str">
+        <v/>
+      </c>
+      <c r="R81">
+        <v>100</v>
+      </c>
+      <c r="S81" t="str">
+        <v/>
+      </c>
+      <c r="T81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B82" t="str">
+        <v>ก23106</v>
+      </c>
+      <c r="C82" t="str">
+        <v>ลูกเสือ-เนตรนารี 2</v>
+      </c>
+      <c r="D82">
+        <v>20</v>
+      </c>
+      <c r="E82" t="str">
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F82" t="str">
+        <v/>
+      </c>
+      <c r="G82" t="str">
+        <v/>
+      </c>
+      <c r="H82" t="str">
+        <v/>
+      </c>
+      <c r="I82" t="str">
+        <v/>
+      </c>
+      <c r="J82" t="str">
+        <v/>
+      </c>
+      <c r="K82" t="str">
+        <v/>
+      </c>
+      <c r="L82" t="str">
+        <v/>
+      </c>
+      <c r="M82" t="str">
+        <v/>
+      </c>
+      <c r="N82" t="str">
+        <v/>
+      </c>
+      <c r="O82" t="str">
+        <v/>
+      </c>
+      <c r="P82" t="str">
+        <v/>
+      </c>
+      <c r="Q82" t="str">
+        <v/>
+      </c>
+      <c r="R82">
+        <v>100</v>
+      </c>
+      <c r="S82" t="str">
+        <v/>
+      </c>
+      <c r="T82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B83" t="str">
+        <v>ก23103</v>
+      </c>
+      <c r="C83" t="str">
+        <v>ชุมนุม 1</v>
+      </c>
+      <c r="D83">
+        <v>13</v>
+      </c>
+      <c r="E83" t="str">
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F83" t="str">
+        <v/>
+      </c>
+      <c r="G83" t="str">
+        <v/>
+      </c>
+      <c r="H83" t="str">
+        <v/>
+      </c>
+      <c r="I83" t="str">
+        <v/>
+      </c>
+      <c r="J83" t="str">
+        <v/>
+      </c>
+      <c r="K83" t="str">
+        <v/>
+      </c>
+      <c r="L83" t="str">
+        <v/>
+      </c>
+      <c r="M83" t="str">
+        <v/>
+      </c>
+      <c r="N83" t="str">
+        <v/>
+      </c>
+      <c r="O83" t="str">
+        <v/>
+      </c>
+      <c r="P83" t="str">
+        <v/>
+      </c>
+      <c r="Q83" t="str">
+        <v/>
+      </c>
+      <c r="R83">
+        <v>100</v>
+      </c>
+      <c r="S83" t="str">
+        <v/>
+      </c>
+      <c r="T83">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B84" t="str">
+        <v>ก23107</v>
+      </c>
+      <c r="C84" t="str">
+        <v>ชุมนุม 2</v>
+      </c>
+      <c r="D84">
+        <v>12</v>
+      </c>
+      <c r="E84" t="str">
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F84" t="str">
+        <v/>
+      </c>
+      <c r="G84" t="str">
+        <v/>
+      </c>
+      <c r="H84" t="str">
+        <v/>
+      </c>
+      <c r="I84" t="str">
+        <v/>
+      </c>
+      <c r="J84" t="str">
+        <v/>
+      </c>
+      <c r="K84" t="str">
+        <v/>
+      </c>
+      <c r="L84" t="str">
+        <v/>
+      </c>
+      <c r="M84" t="str">
+        <v/>
+      </c>
+      <c r="N84" t="str">
+        <v/>
+      </c>
+      <c r="O84" t="str">
+        <v/>
+      </c>
+      <c r="P84" t="str">
+        <v/>
+      </c>
+      <c r="Q84" t="str">
+        <v/>
+      </c>
+      <c r="R84">
+        <v>100</v>
+      </c>
+      <c r="S84" t="str">
+        <v/>
+      </c>
+      <c r="T84">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B85" t="str">
         <v>ก23104</v>
       </c>
-      <c r="C74" t="str">
-        <v>กิจกรรมเพื่อสังคมและสาธารณประโยชน์</v>
-      </c>
-      <c r="D74">
-        <v>15</v>
-      </c>
-      <c r="E74" t="str">
+      <c r="C85" t="str">
+        <v>กิจกรรมเพื่อสังคมและสาธารณประโยชน์ 1</v>
+      </c>
+      <c r="D85">
+        <v>7</v>
+      </c>
+      <c r="E85" t="str">
         <v>กิจกรรม</v>
       </c>
-      <c r="F74" t="str">
-        <v/>
-      </c>
-      <c r="G74" t="str">
-        <v/>
-      </c>
-      <c r="H74" t="str">
-        <v/>
-      </c>
-      <c r="I74" t="str">
-        <v/>
-      </c>
-      <c r="J74" t="str">
-        <v/>
-      </c>
-      <c r="K74" t="str">
-        <v/>
-      </c>
-      <c r="L74" t="str">
-        <v/>
-      </c>
-      <c r="M74" t="str">
-        <v/>
-      </c>
-      <c r="N74" t="str">
-        <v/>
-      </c>
-      <c r="O74" t="str">
-        <v/>
-      </c>
-      <c r="P74" t="str">
-        <v/>
-      </c>
-      <c r="Q74" t="str">
-        <v/>
-      </c>
-      <c r="R74">
-        <v>100</v>
-      </c>
-      <c r="S74" t="str">
-        <v/>
-      </c>
-      <c r="T74" t="str">
-        <v/>
+      <c r="F85" t="str">
+        <v/>
+      </c>
+      <c r="G85" t="str">
+        <v/>
+      </c>
+      <c r="H85" t="str">
+        <v/>
+      </c>
+      <c r="I85" t="str">
+        <v/>
+      </c>
+      <c r="J85" t="str">
+        <v/>
+      </c>
+      <c r="K85" t="str">
+        <v/>
+      </c>
+      <c r="L85" t="str">
+        <v/>
+      </c>
+      <c r="M85" t="str">
+        <v/>
+      </c>
+      <c r="N85" t="str">
+        <v/>
+      </c>
+      <c r="O85" t="str">
+        <v/>
+      </c>
+      <c r="P85" t="str">
+        <v/>
+      </c>
+      <c r="Q85" t="str">
+        <v/>
+      </c>
+      <c r="R85">
+        <v>100</v>
+      </c>
+      <c r="S85" t="str">
+        <v/>
+      </c>
+      <c r="T85">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>ม.3</v>
+      </c>
+      <c r="B86" t="str">
+        <v>ก23108</v>
+      </c>
+      <c r="C86" t="str">
+        <v>กิจกรรมเพื่อสังคมและสาธารณประโยชน์ 2</v>
+      </c>
+      <c r="D86">
+        <v>8</v>
+      </c>
+      <c r="E86" t="str">
+        <v>กิจกรรม</v>
+      </c>
+      <c r="F86" t="str">
+        <v/>
+      </c>
+      <c r="G86" t="str">
+        <v/>
+      </c>
+      <c r="H86" t="str">
+        <v/>
+      </c>
+      <c r="I86" t="str">
+        <v/>
+      </c>
+      <c r="J86" t="str">
+        <v/>
+      </c>
+      <c r="K86" t="str">
+        <v/>
+      </c>
+      <c r="L86" t="str">
+        <v/>
+      </c>
+      <c r="M86" t="str">
+        <v/>
+      </c>
+      <c r="N86" t="str">
+        <v/>
+      </c>
+      <c r="O86" t="str">
+        <v/>
+      </c>
+      <c r="P86" t="str">
+        <v/>
+      </c>
+      <c r="Q86" t="str">
+        <v/>
+      </c>
+      <c r="R86">
+        <v>100</v>
+      </c>
+      <c r="S86" t="str">
+        <v/>
+      </c>
+      <c r="T86">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -5018,7 +5762,7 @@
     <mergeCell ref="P1:R1"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T86"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5137,12 +5881,12 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>กิจกรรมพัฒนาผู้เรียน (120 ชม./ปี): แนะแนว 40, ลูกเสือ-เนตรนารี 40, ชุมนุม 25, กิจกรรมเพื่อสังคมและสาธารณประโยชน์ 15</v>
+        <v>กิจกรรมพัฒนาผู้เรียน (120 ชม./ปี = ภาคละ 60): แนะแนว 20+20, ลูกเสือ-เนตรนารี 20+20, ชุมนุม 13+12, กิจกรรมเพื่อสังคมและสาธารณประโยชน์ 7+8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>• กิจกรรมประเมินผ่าน/ไม่ผ่านเป็นรายปีในหน้า "ประเมินกิจกรรม" จึงเว้นช่องภาคเรียนและช่องคะแนนไว้</v>
+        <v>• กิจกรรมแยกภาค 1 / ภาค 2 เหมือนวิชาอื่น (รหัส 01–04 = ภาค 1, 05–08 = ภาค 2) ประเมินผ่าน/ไม่ผ่านรายภาคในหน้า "ประเมินกิจกรรม" ไม่มีคะแนน</v>
       </c>
     </row>
     <row r="24">

</xml_diff>